<commit_message>
data(cf-consulting): add sample team data to Practice Tracker
Team members:
- Rino Raj (Team Lead) - Client-Facing Lead pathway
- John Joseph (Project Lead) - Technical Assessor pathway
- Nandu S (Team Lead) - Lucee Specialist pathway
- Rehnasha RS (Software Engineer) - UI/API Specialist pathway
- Renjith M (Tech Lead) - Performance Specialist pathway
- Lajin M J (Architect, TAM) - Modernization Architect pathway
- Shilpa S (Senior Engineer) - AI Integration Advisor pathway

Includes readiness assessment sample data across all 5 categories.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/engineering-academy/cf-consulting/ASSESSMENT/CF_Consulting_Practice_Tracker.xlsx
+++ b/engineering-academy/cf-consulting/ASSESSMENT/CF_Consulting_Practice_Tracker.xlsx
@@ -532,94 +532,338 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Client-Facing Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Modernization Architect</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>John Joseph</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Project Lead</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Technical Assessor</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Client-Facing Lead</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Nandu S</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Team Lead</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Lucee Specialist</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Specialist</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Rehnasha RS</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>UI/API Specialist</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Renjith M</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Performance Specialist</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Technical Assessor</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Lajin M J</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Architect, TAM</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Modernization Architect</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Client-Facing Lead</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Shilpa S</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Senior Engineer</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>AI Integration Advisor</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
       <c r="K10" s="3" t="n"/>
     </row>
     <row r="11">
@@ -815,93 +1059,333 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Assessment and Discovery</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>I can review a legacy CF application and produce a structured assessment report.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Assessment and Discovery</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>I can lead a 2-hour discovery session with a client.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Assessment and Discovery</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>I can identify technical risks and communicate them clearly.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Ready with Support</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Architecture and Modernization</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>I can recommend a modernization path with clear rationale.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Architecture and Modernization</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>I can design a target architecture for a CF modernization engagement.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Ready with Support</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Client Communication</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>I can explain technical concepts to non-technical stakeholders.</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Client Communication</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>I can communicate risks early without alarming clients.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Estimation and Proposal</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>I can produce a WBS and estimate effort for a CF project.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Ready with Support</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Estimation and Proposal</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>I can write clear scope statements and assumptions for a proposal.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Ready with Support</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Specialist Capabilities</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>I can plan and execute a Lucee migration.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Existing project work</t>
+        </is>
+      </c>
       <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
@@ -1130,34 +1614,124 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Client-Facing Lead</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Lead real client discovery session</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Complete Phase 9 exercises, shadow 2 discovery sessions</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>John Joseph</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Technical Assessor</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Complete 3 legacy assessments</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Practice with BlogCFC5 scenario</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Shilpa S</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>AI Integration Advisor</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Build AI use case analysis capability</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Complete Phase 6 capstone exercise</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -1354,67 +1928,239 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Observer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Legacy Assessment</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Can review a legacy CF application</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>BlogCFC5 practice</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Legacy Assessment</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Can contribute to assessment with review</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>5 real client sessions</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Legacy Assessment</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Can lead assessment with peer review</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>3 migrations completed</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Legacy Assessment</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Can own client assessment end-to-end</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Observer</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Can attend discovery session</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
       <c r="F8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Can contribute to discovery with review</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
       <c r="F9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Can lead discovery session</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
       <c r="F10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Can mentor others in discovery</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="F11" s="3" t="n"/>
     </row>
     <row r="12">
@@ -1683,24 +2429,84 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>John Joseph</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>BlogCFC5 Assessment</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Good questioning technique, clear summary</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Needs more practice on time management</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Lajin M J</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Nandu S</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Architecture diagram review</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Clear visuals</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -1981,28 +2787,104 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Summit Manufacturing</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Discovery Workshop</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Positive - moving to proposal</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Professional, good listener</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Supported Lead</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>BlogCFC5 scenario</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Summit Manufacturing</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Legacy Assessment</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>John Joseph</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Thorough report</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Contributor</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>CF9 app review</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -2308,22 +3190,78 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Month 1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Lead discovery session</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Completed 2 discovery exercises</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Limited real client exposure</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Shadow real client meeting</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>John Joseph</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>John Joseph</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Goal: Complete readiness check</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Finished self-assessment</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Start BlogCFC5 exercise</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Rino Raj</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -2573,14 +3511,42 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Lajin M J</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Modernization Architect</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>5+ modernization projects delivered</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>

</xml_diff>